<commit_message>
ran Kaihalulu 2026-02-28 both parts
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A58CEEF-8FAD-41FC-92A5-EE8C1CECE8B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0270C34-53F2-404B-8242-FEAFF57DCE87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15585" yWindow="720" windowWidth="13215" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="113">
   <si>
     <t>Date</t>
   </si>
@@ -369,6 +369,9 @@
   </si>
   <si>
     <t>same CRM opened 02/23/2026</t>
+  </si>
+  <si>
+    <t>second run of day, same CRM opened 02/23/2026</t>
   </si>
 </sst>
 </file>
@@ -1205,7 +1208,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G309"/>
+  <dimension ref="A1:G311"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -7509,7 +7512,7 @@
         <v>2212.31</v>
       </c>
       <c r="D309">
-        <f t="shared" ref="D309" si="11">100*(B309-C309)/C309</f>
+        <f t="shared" ref="D309:D310" si="11">100*(B309-C309)/C309</f>
         <v>-0.45193530743881938</v>
       </c>
       <c r="E309">
@@ -7517,6 +7520,48 @@
       </c>
       <c r="F309" t="s">
         <v>111</v>
+      </c>
+    </row>
+    <row r="310" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A310" s="1">
+        <v>46089</v>
+      </c>
+      <c r="B310" s="4">
+        <v>2207.98432</v>
+      </c>
+      <c r="C310">
+        <v>2212.31</v>
+      </c>
+      <c r="D310">
+        <f t="shared" si="11"/>
+        <v>-0.19552775153572149</v>
+      </c>
+      <c r="E310">
+        <v>217</v>
+      </c>
+      <c r="F310" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="311" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A311" s="1">
+        <v>46089</v>
+      </c>
+      <c r="B311" s="4">
+        <v>2203.7444399999999</v>
+      </c>
+      <c r="C311">
+        <v>2212.31</v>
+      </c>
+      <c r="D311">
+        <f t="shared" ref="D311" si="12">100*(B311-C311)/C311</f>
+        <v>-0.38717720391807681</v>
+      </c>
+      <c r="E311">
+        <v>217</v>
+      </c>
+      <c r="F311" t="s">
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MP add data first run 3/15/26
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0270C34-53F2-404B-8242-FEAFF57DCE87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0572EECB-52BD-43A5-B49F-D0E42B2F3989}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15585" yWindow="720" windowWidth="13215" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="113">
   <si>
     <t>Date</t>
   </si>
@@ -1208,7 +1208,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G311"/>
+  <dimension ref="A1:G313"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -7564,6 +7564,48 @@
         <v>112</v>
       </c>
     </row>
+    <row r="312" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A312" s="1">
+        <v>46094</v>
+      </c>
+      <c r="B312" s="4">
+        <v>2209.9749200000001</v>
+      </c>
+      <c r="C312">
+        <v>2212.31</v>
+      </c>
+      <c r="D312">
+        <f>100*(B312-C312)/C312</f>
+        <v>-0.1055494031125762</v>
+      </c>
+      <c r="E312">
+        <v>217</v>
+      </c>
+      <c r="F312" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="313" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A313" s="1">
+        <v>46096</v>
+      </c>
+      <c r="B313" s="4">
+        <v>2195.19785</v>
+      </c>
+      <c r="C313">
+        <v>2212.31</v>
+      </c>
+      <c r="D313">
+        <f>100*(B313-C313)/C313</f>
+        <v>-0.77349693306995537</v>
+      </c>
+      <c r="E313">
+        <v>217</v>
+      </c>
+      <c r="F313" t="s">
+        <v>111</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
mp adding run 6 7 8 respo titrations
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{532036C2-4169-4557-9EAD-E4B39D926936}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94A18072-EAC2-4FFC-81F2-B5E77EB56606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15585" yWindow="720" windowWidth="13215" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15270" yWindow="1410" windowWidth="13215" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="113">
   <si>
     <t>Date</t>
   </si>
@@ -1208,7 +1208,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G314"/>
+  <dimension ref="A1:G315"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -7627,6 +7627,27 @@
         <v>111</v>
       </c>
     </row>
+    <row r="315" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A315" s="1">
+        <v>46098</v>
+      </c>
+      <c r="B315" s="4">
+        <v>2209.22534</v>
+      </c>
+      <c r="C315">
+        <v>2212.31</v>
+      </c>
+      <c r="D315">
+        <f>100*(B315-C315)/C315</f>
+        <v>-0.13943163480705623</v>
+      </c>
+      <c r="E315">
+        <v>217</v>
+      </c>
+      <c r="F315" t="s">
+        <v>111</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Adding all TA calculated data from runs so far
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94A18072-EAC2-4FFC-81F2-B5E77EB56606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{435FF5C8-4991-4239-87E3-BA9C1EA1D3D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15270" yWindow="1410" windowWidth="13215" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15540" yWindow="1020" windowWidth="13215" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="113">
   <si>
     <t>Date</t>
   </si>
@@ -1208,7 +1208,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G315"/>
+  <dimension ref="A1:G316"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -7648,6 +7648,27 @@
         <v>111</v>
       </c>
     </row>
+    <row r="316" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A316" s="1">
+        <v>46100</v>
+      </c>
+      <c r="B316" s="4">
+        <v>2203.9237600000001</v>
+      </c>
+      <c r="C316">
+        <v>2213.31</v>
+      </c>
+      <c r="D316">
+        <f>100*(B316-C316)/C316</f>
+        <v>-0.42408157917326611</v>
+      </c>
+      <c r="E316">
+        <v>217</v>
+      </c>
+      <c r="F316" t="s">
+        <v>111</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
MP add biofac respo run 12 13 14 data
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{435FF5C8-4991-4239-87E3-BA9C1EA1D3D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FE4AA8C-8BBA-425E-997D-7AA67767506D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15540" yWindow="1020" windowWidth="13215" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="114">
   <si>
     <t>Date</t>
   </si>
@@ -372,6 +372,9 @@
   </si>
   <si>
     <t>second run of day, same CRM opened 02/23/2026</t>
+  </si>
+  <si>
+    <t>new CRM opened 03/20/2026</t>
   </si>
 </sst>
 </file>
@@ -1208,7 +1211,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G316"/>
+  <dimension ref="A1:G318"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -7656,17 +7659,59 @@
         <v>2203.9237600000001</v>
       </c>
       <c r="C316">
-        <v>2213.31</v>
+        <v>2212.31</v>
       </c>
       <c r="D316">
         <f>100*(B316-C316)/C316</f>
-        <v>-0.42408157917326611</v>
+        <v>-0.37907164909076108</v>
       </c>
       <c r="E316">
         <v>217</v>
       </c>
       <c r="F316" t="s">
         <v>111</v>
+      </c>
+    </row>
+    <row r="317" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A317" s="1">
+        <v>46101</v>
+      </c>
+      <c r="B317" s="4">
+        <v>2248.6597999999999</v>
+      </c>
+      <c r="C317">
+        <v>2212.31</v>
+      </c>
+      <c r="D317">
+        <f>100*(B317-C317)/C317</f>
+        <v>1.6430699133484892</v>
+      </c>
+      <c r="E317">
+        <v>217</v>
+      </c>
+      <c r="F317" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="318" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A318" s="1">
+        <v>46101</v>
+      </c>
+      <c r="B318" s="4">
+        <v>2210.7517400000002</v>
+      </c>
+      <c r="C318">
+        <v>2212.31</v>
+      </c>
+      <c r="D318">
+        <f>100*(B318-C318)/C318</f>
+        <v>-7.0435879239337668E-2</v>
+      </c>
+      <c r="E318">
+        <v>217</v>
+      </c>
+      <c r="F318" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mica ran Maya's respo reruns from 3/25/2026
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FE4AA8C-8BBA-425E-997D-7AA67767506D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFC6D407-AA4E-4174-9788-AC7D555FD5CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15540" yWindow="1020" windowWidth="13215" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15585" yWindow="900" windowWidth="13215" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="114">
   <si>
     <t>Date</t>
   </si>
@@ -1211,7 +1211,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G318"/>
+  <dimension ref="A1:G319"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -7578,7 +7578,7 @@
         <v>2212.31</v>
       </c>
       <c r="D312">
-        <f>100*(B312-C312)/C312</f>
+        <f t="shared" ref="D312:D319" si="13">100*(B312-C312)/C312</f>
         <v>-0.1055494031125762</v>
       </c>
       <c r="E312">
@@ -7599,7 +7599,7 @@
         <v>2212.31</v>
       </c>
       <c r="D313">
-        <f>100*(B313-C313)/C313</f>
+        <f t="shared" si="13"/>
         <v>-0.77349693306995537</v>
       </c>
       <c r="E313">
@@ -7620,7 +7620,7 @@
         <v>2212.31</v>
       </c>
       <c r="D314">
-        <f>100*(B314-C314)/C314</f>
+        <f t="shared" si="13"/>
         <v>0.45898947254227468</v>
       </c>
       <c r="E314">
@@ -7641,7 +7641,7 @@
         <v>2212.31</v>
       </c>
       <c r="D315">
-        <f>100*(B315-C315)/C315</f>
+        <f t="shared" si="13"/>
         <v>-0.13943163480705623</v>
       </c>
       <c r="E315">
@@ -7662,7 +7662,7 @@
         <v>2212.31</v>
       </c>
       <c r="D316">
-        <f>100*(B316-C316)/C316</f>
+        <f t="shared" si="13"/>
         <v>-0.37907164909076108</v>
       </c>
       <c r="E316">
@@ -7683,7 +7683,7 @@
         <v>2212.31</v>
       </c>
       <c r="D317">
-        <f>100*(B317-C317)/C317</f>
+        <f t="shared" si="13"/>
         <v>1.6430699133484892</v>
       </c>
       <c r="E317">
@@ -7704,13 +7704,34 @@
         <v>2212.31</v>
       </c>
       <c r="D318">
-        <f>100*(B318-C318)/C318</f>
+        <f t="shared" si="13"/>
         <v>-7.0435879239337668E-2</v>
       </c>
       <c r="E318">
         <v>217</v>
       </c>
       <c r="F318" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="319" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A319" s="1">
+        <v>46108</v>
+      </c>
+      <c r="B319" s="4">
+        <v>2205.7238900000002</v>
+      </c>
+      <c r="C319">
+        <v>2212.31</v>
+      </c>
+      <c r="D319">
+        <f t="shared" si="13"/>
+        <v>-0.29770285357837445</v>
+      </c>
+      <c r="E319">
+        <v>217</v>
+      </c>
+      <c r="F319" t="s">
         <v>113</v>
       </c>
     </row>

</xml_diff>

<commit_message>
dmb prelim exp TA data
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFC6D407-AA4E-4174-9788-AC7D555FD5CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{287AAF7E-0A38-45A2-9633-511112920C5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15585" yWindow="900" windowWidth="13215" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9150" yWindow="1500" windowWidth="13215" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="115">
   <si>
     <t>Date</t>
   </si>
@@ -375,6 +375,9 @@
   </si>
   <si>
     <t>new CRM opened 03/20/2026</t>
+  </si>
+  <si>
+    <t>same CRM opened 03/20/2026</t>
   </si>
 </sst>
 </file>
@@ -1211,7 +1214,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G319"/>
+  <dimension ref="A1:G320"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -7578,7 +7581,7 @@
         <v>2212.31</v>
       </c>
       <c r="D312">
-        <f t="shared" ref="D312:D319" si="13">100*(B312-C312)/C312</f>
+        <f t="shared" ref="D312:D320" si="13">100*(B312-C312)/C312</f>
         <v>-0.1055494031125762</v>
       </c>
       <c r="E312">
@@ -7733,6 +7736,27 @@
       </c>
       <c r="F319" t="s">
         <v>113</v>
+      </c>
+    </row>
+    <row r="320" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A320" s="1">
+        <v>46119</v>
+      </c>
+      <c r="B320">
+        <v>2206.0186037397002</v>
+      </c>
+      <c r="C320">
+        <v>2212.31</v>
+      </c>
+      <c r="D320">
+        <f t="shared" si="13"/>
+        <v>-0.28438131456711468</v>
+      </c>
+      <c r="E320">
+        <v>217</v>
+      </c>
+      <c r="F320" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MP adding Biofac April 6 12pm samples
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{287AAF7E-0A38-45A2-9633-511112920C5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BE1AFC4-7391-4DA6-989D-DA4C8AC08C5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9150" yWindow="1500" windowWidth="13215" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11100" yWindow="780" windowWidth="20355" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="115">
   <si>
     <t>Date</t>
   </si>
@@ -1214,13 +1214,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G320"/>
+  <dimension ref="A1:G321"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="14.42578125" customWidth="1"/>
     <col min="3" max="3" width="14.7109375" customWidth="1"/>
-    <col min="6" max="6" width="24.140625" customWidth="1"/>
+    <col min="6" max="6" width="30.140625" customWidth="1"/>
     <col min="14" max="14" width="9" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7581,7 +7581,7 @@
         <v>2212.31</v>
       </c>
       <c r="D312">
-        <f t="shared" ref="D312:D320" si="13">100*(B312-C312)/C312</f>
+        <f t="shared" ref="D312:D321" si="13">100*(B312-C312)/C312</f>
         <v>-0.1055494031125762</v>
       </c>
       <c r="E312">
@@ -7735,7 +7735,7 @@
         <v>217</v>
       </c>
       <c r="F319" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="320" spans="1:6" x14ac:dyDescent="0.25">
@@ -7756,6 +7756,27 @@
         <v>217</v>
       </c>
       <c r="F320" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="321" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A321" s="1">
+        <v>46133</v>
+      </c>
+      <c r="B321" s="4">
+        <v>2200.2290600000001</v>
+      </c>
+      <c r="C321">
+        <v>2212.31</v>
+      </c>
+      <c r="D321">
+        <f t="shared" si="13"/>
+        <v>-0.54607808128154856</v>
+      </c>
+      <c r="E321">
+        <v>217</v>
+      </c>
+      <c r="F321" t="s">
         <v>114</v>
       </c>
     </row>

</xml_diff>

<commit_message>
powell respo run 16 17 18
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BE1AFC4-7391-4DA6-989D-DA4C8AC08C5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13BFCE0E-E099-46F8-9756-87857A5B1348}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11100" yWindow="780" windowWidth="20355" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6990" yWindow="435" windowWidth="20355" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="115">
   <si>
     <t>Date</t>
   </si>
@@ -1214,7 +1214,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G321"/>
+  <dimension ref="A1:G322"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -7581,7 +7581,7 @@
         <v>2212.31</v>
       </c>
       <c r="D312">
-        <f t="shared" ref="D312:D321" si="13">100*(B312-C312)/C312</f>
+        <f t="shared" ref="D312:D322" si="13">100*(B312-C312)/C312</f>
         <v>-0.1055494031125762</v>
       </c>
       <c r="E312">
@@ -7777,6 +7777,27 @@
         <v>217</v>
       </c>
       <c r="F321" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="322" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A322" s="1">
+        <v>46146</v>
+      </c>
+      <c r="B322" s="2">
+        <v>2209.3617300000001</v>
+      </c>
+      <c r="C322">
+        <v>2212.31</v>
+      </c>
+      <c r="D322">
+        <f t="shared" si="13"/>
+        <v>-0.13326658560508545</v>
+      </c>
+      <c r="E322">
+        <v>217</v>
+      </c>
+      <c r="F322" t="s">
         <v>114</v>
       </c>
     </row>

</xml_diff>

<commit_message>
powell ta respo runs 19 20 21 22 23 24
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13BFCE0E-E099-46F8-9756-87857A5B1348}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A374D170-86BE-459D-967D-384BED68D6D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6990" yWindow="435" windowWidth="20355" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7965" yWindow="600" windowWidth="20355" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="118">
   <si>
     <t>Date</t>
   </si>
@@ -378,6 +378,15 @@
   </si>
   <si>
     <t>same CRM opened 03/20/2026</t>
+  </si>
+  <si>
+    <t>new CRM opened 05/04/2026, finished CRM above</t>
+  </si>
+  <si>
+    <t>same CRM opened 05/04/2026, MP added to end of run as 47th sample and looks great yay!</t>
+  </si>
+  <si>
+    <t>same CRM opened 05/04/2026</t>
   </si>
 </sst>
 </file>
@@ -1214,7 +1223,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G322"/>
+  <dimension ref="A1:G325"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -7581,7 +7590,7 @@
         <v>2212.31</v>
       </c>
       <c r="D312">
-        <f t="shared" ref="D312:D322" si="13">100*(B312-C312)/C312</f>
+        <f t="shared" ref="D312:D325" si="13">100*(B312-C312)/C312</f>
         <v>-0.1055494031125762</v>
       </c>
       <c r="E312">
@@ -7799,6 +7808,69 @@
       </c>
       <c r="F322" t="s">
         <v>114</v>
+      </c>
+    </row>
+    <row r="323" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A323" s="1">
+        <v>46146</v>
+      </c>
+      <c r="B323" s="2">
+        <v>2211.4530599999998</v>
+      </c>
+      <c r="C323">
+        <v>2212.31</v>
+      </c>
+      <c r="D323">
+        <f t="shared" si="13"/>
+        <v>-3.8735077814597521E-2</v>
+      </c>
+      <c r="E323">
+        <v>217</v>
+      </c>
+      <c r="F323" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="324" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A324" s="1">
+        <v>46146</v>
+      </c>
+      <c r="B324" s="2">
+        <v>2207.8857499999999</v>
+      </c>
+      <c r="C324">
+        <v>2212.31</v>
+      </c>
+      <c r="D324">
+        <f t="shared" si="13"/>
+        <v>-0.19998327539992267</v>
+      </c>
+      <c r="E324">
+        <v>217</v>
+      </c>
+      <c r="F324" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="325" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A325" s="1">
+        <v>46147</v>
+      </c>
+      <c r="B325" s="2">
+        <v>2218.4741899999999</v>
+      </c>
+      <c r="C325">
+        <v>2212.31</v>
+      </c>
+      <c r="D325">
+        <f t="shared" si="13"/>
+        <v>0.27863138529410264</v>
+      </c>
+      <c r="E325">
+        <v>217</v>
+      </c>
+      <c r="F325" t="s">
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MC ran Sandy 2026-05-02
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A374D170-86BE-459D-967D-384BED68D6D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C023F88A-97E6-47CD-A9FA-F60F53445FAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7965" yWindow="600" windowWidth="20355" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15240" yWindow="945" windowWidth="13425" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="119">
   <si>
     <t>Date</t>
   </si>
@@ -387,6 +387,9 @@
   </si>
   <si>
     <t>same CRM opened 05/04/2026</t>
+  </si>
+  <si>
+    <t>same CRM opened 05/04/2026, MC ran before second run of the day</t>
   </si>
 </sst>
 </file>
@@ -1223,7 +1226,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G325"/>
+  <dimension ref="A1:G327"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -7590,7 +7593,7 @@
         <v>2212.31</v>
       </c>
       <c r="D312">
-        <f t="shared" ref="D312:D325" si="13">100*(B312-C312)/C312</f>
+        <f t="shared" ref="D312:D327" si="13">100*(B312-C312)/C312</f>
         <v>-0.1055494031125762</v>
       </c>
       <c r="E312">
@@ -7871,6 +7874,48 @@
       </c>
       <c r="F325" t="s">
         <v>117</v>
+      </c>
+    </row>
+    <row r="326" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A326" s="1">
+        <v>46149</v>
+      </c>
+      <c r="B326" s="4">
+        <v>2209.5682700000002</v>
+      </c>
+      <c r="C326">
+        <v>2212.31</v>
+      </c>
+      <c r="D326">
+        <f t="shared" si="13"/>
+        <v>-0.1239306426314456</v>
+      </c>
+      <c r="E326">
+        <v>217</v>
+      </c>
+      <c r="F326" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="327" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A327" s="1">
+        <v>46149</v>
+      </c>
+      <c r="B327" s="4">
+        <v>2211.0061500000002</v>
+      </c>
+      <c r="C327">
+        <v>2212.31</v>
+      </c>
+      <c r="D327">
+        <f t="shared" si="13"/>
+        <v>-5.8936134628500704E-2</v>
+      </c>
+      <c r="E327">
+        <v>217</v>
+      </c>
+      <c r="F327" t="s">
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
powell biofac respo run 25 26
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C023F88A-97E6-47CD-A9FA-F60F53445FAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C56BC9C0-B717-4FD7-83B9-741E50D6A9FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15240" yWindow="945" windowWidth="13425" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="2100" windowWidth="13425" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="120">
   <si>
     <t>Date</t>
   </si>
@@ -390,6 +390,9 @@
   </si>
   <si>
     <t>same CRM opened 05/04/2026, MC ran before second run of the day</t>
+  </si>
+  <si>
+    <t>same CRM opened 05/04/2026, re-run because above was BAD</t>
   </si>
 </sst>
 </file>
@@ -556,7 +559,7 @@
       <family val="3"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -736,8 +739,14 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -852,6 +861,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFD6DADC"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -897,13 +915,16 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1226,7 +1247,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G327"/>
+  <dimension ref="A1:G329"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -7782,7 +7803,7 @@
         <v>2212.31</v>
       </c>
       <c r="D321">
-        <f t="shared" si="13"/>
+        <f>100*(B321-C321)/C321</f>
         <v>-0.54607808128154856</v>
       </c>
       <c r="E321">
@@ -7803,7 +7824,7 @@
         <v>2212.31</v>
       </c>
       <c r="D322">
-        <f t="shared" si="13"/>
+        <f t="shared" ref="D322:D328" si="14">100*(B322-C322)/C322</f>
         <v>-0.13326658560508545</v>
       </c>
       <c r="E322">
@@ -7824,7 +7845,7 @@
         <v>2212.31</v>
       </c>
       <c r="D323">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>-3.8735077814597521E-2</v>
       </c>
       <c r="E323">
@@ -7845,7 +7866,7 @@
         <v>2212.31</v>
       </c>
       <c r="D324">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>-0.19998327539992267</v>
       </c>
       <c r="E324">
@@ -7866,7 +7887,7 @@
         <v>2212.31</v>
       </c>
       <c r="D325">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0.27863138529410264</v>
       </c>
       <c r="E325">
@@ -7887,7 +7908,7 @@
         <v>2212.31</v>
       </c>
       <c r="D326">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>-0.1239306426314456</v>
       </c>
       <c r="E326">
@@ -7908,7 +7929,7 @@
         <v>2212.31</v>
       </c>
       <c r="D327">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>-5.8936134628500704E-2</v>
       </c>
       <c r="E327">
@@ -7916,6 +7937,48 @@
       </c>
       <c r="F327" t="s">
         <v>118</v>
+      </c>
+    </row>
+    <row r="328" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A328" s="1">
+        <v>46150</v>
+      </c>
+      <c r="B328" s="5">
+        <v>2237.4041499999998</v>
+      </c>
+      <c r="C328">
+        <v>2212.31</v>
+      </c>
+      <c r="D328">
+        <f>100*(B328-C328)/C328</f>
+        <v>1.1342962785504698</v>
+      </c>
+      <c r="E328">
+        <v>217</v>
+      </c>
+      <c r="F328" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="329" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A329" s="1">
+        <v>46150</v>
+      </c>
+      <c r="B329" s="2">
+        <v>2211.5893000000001</v>
+      </c>
+      <c r="C329">
+        <v>2212.31</v>
+      </c>
+      <c r="D329">
+        <f>100*(B329-C329)/C329</f>
+        <v>-3.2576808855895041E-2</v>
+      </c>
+      <c r="E329">
+        <v>217</v>
+      </c>
+      <c r="F329" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
powell respo run 27 28
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C56BC9C0-B717-4FD7-83B9-741E50D6A9FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBB84603-E91C-4057-80B0-44F3056ED4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="2100" windowWidth="13425" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15240" yWindow="945" windowWidth="13425" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="120">
   <si>
     <t>Date</t>
   </si>
@@ -1247,7 +1247,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G329"/>
+  <dimension ref="A1:G330"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -7614,7 +7614,7 @@
         <v>2212.31</v>
       </c>
       <c r="D312">
-        <f t="shared" ref="D312:D327" si="13">100*(B312-C312)/C312</f>
+        <f t="shared" ref="D312:D320" si="13">100*(B312-C312)/C312</f>
         <v>-0.1055494031125762</v>
       </c>
       <c r="E312">
@@ -7824,7 +7824,7 @@
         <v>2212.31</v>
       </c>
       <c r="D322">
-        <f t="shared" ref="D322:D328" si="14">100*(B322-C322)/C322</f>
+        <f t="shared" ref="D322:D327" si="14">100*(B322-C322)/C322</f>
         <v>-0.13326658560508545</v>
       </c>
       <c r="E322">
@@ -7979,6 +7979,27 @@
       </c>
       <c r="F329" t="s">
         <v>119</v>
+      </c>
+    </row>
+    <row r="330" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A330" s="1">
+        <v>46154</v>
+      </c>
+      <c r="B330" s="2">
+        <v>2193.0488700000001</v>
+      </c>
+      <c r="C330">
+        <v>2212.31</v>
+      </c>
+      <c r="D330">
+        <f>100*(B330-C330)/C330</f>
+        <v>-0.87063431435919314</v>
+      </c>
+      <c r="E330">
+        <v>217</v>
+      </c>
+      <c r="F330" t="s">
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
POWELL BIOFAC ADD APRIL 7 0000 AND RENAME APRIL 6 1200
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBB84603-E91C-4057-80B0-44F3056ED4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB67A650-804D-4A4E-B435-4A3761182E2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15240" yWindow="945" windowWidth="13425" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14040" yWindow="1095" windowWidth="14805" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="121">
   <si>
     <t>Date</t>
   </si>
@@ -393,6 +393,9 @@
   </si>
   <si>
     <t>same CRM opened 05/04/2026, re-run because above was BAD</t>
+  </si>
+  <si>
+    <t>new CRM opened 5/14/2026 (above CRM not enough for redo)</t>
   </si>
 </sst>
 </file>
@@ -1247,7 +1250,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G330"/>
+  <dimension ref="A1:G332"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -8002,6 +8005,48 @@
         <v>117</v>
       </c>
     </row>
+    <row r="331" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A331" s="1">
+        <v>46156</v>
+      </c>
+      <c r="B331" s="2">
+        <v>2238.6710200000002</v>
+      </c>
+      <c r="C331">
+        <v>2212.31</v>
+      </c>
+      <c r="D331">
+        <f>100*(B331-C331)/C331</f>
+        <v>1.1915608572035692</v>
+      </c>
+      <c r="E331">
+        <v>217</v>
+      </c>
+      <c r="F331" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="332" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A332" s="1">
+        <v>46156</v>
+      </c>
+      <c r="B332" s="2">
+        <v>2227.527</v>
+      </c>
+      <c r="C332">
+        <v>2212.31</v>
+      </c>
+      <c r="D332">
+        <f>100*(B332-C332)/C332</f>
+        <v>0.68783307945089511</v>
+      </c>
+      <c r="E332">
+        <v>217</v>
+      </c>
+      <c r="F332" t="s">
+        <v>120</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
POWELL 24HR 0600 4/7/26 TITRATION
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB67A650-804D-4A4E-B435-4A3761182E2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DC6E3EB-3F52-4E5A-9A24-1460CEE3F257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14040" yWindow="1095" windowWidth="14805" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14040" yWindow="1095" windowWidth="13425" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="123">
   <si>
     <t>Date</t>
   </si>
@@ -396,6 +396,12 @@
   </si>
   <si>
     <t>new CRM opened 5/14/2026 (above CRM not enough for redo)</t>
+  </si>
+  <si>
+    <t>same CRM opened 05/14/2026</t>
+  </si>
+  <si>
+    <t>same CRM opened 05/14/2026, REDO</t>
   </si>
 </sst>
 </file>
@@ -1250,7 +1256,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G332"/>
+  <dimension ref="A1:G334"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -8047,6 +8053,48 @@
         <v>120</v>
       </c>
     </row>
+    <row r="333" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A333" s="1">
+        <v>46157</v>
+      </c>
+      <c r="B333" s="2">
+        <v>2244.2035599999999</v>
+      </c>
+      <c r="C333">
+        <v>2212.31</v>
+      </c>
+      <c r="D333">
+        <f>100*(B333-C333)/C333</f>
+        <v>1.4416406380660929</v>
+      </c>
+      <c r="E333">
+        <v>217</v>
+      </c>
+      <c r="F333" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="334" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A334" s="1">
+        <v>46157</v>
+      </c>
+      <c r="B334" s="2">
+        <v>2211.5452100000002</v>
+      </c>
+      <c r="C334">
+        <v>2212.31</v>
+      </c>
+      <c r="D334">
+        <f>100*(B334-C334)/C334</f>
+        <v>-3.4569748362558626E-2</v>
+      </c>
+      <c r="E334">
+        <v>217</v>
+      </c>
+      <c r="F334" t="s">
+        <v>122</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
TITRATION POWELL 04062026 1800
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DC6E3EB-3F52-4E5A-9A24-1460CEE3F257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48B1EBE6-2598-47EF-9A87-798C160BD7E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14040" yWindow="1095" windowWidth="13425" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="123">
   <si>
     <t>Date</t>
   </si>
@@ -1256,7 +1256,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G334"/>
+  <dimension ref="A1:G336"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -7959,7 +7959,7 @@
         <v>2212.31</v>
       </c>
       <c r="D328">
-        <f>100*(B328-C328)/C328</f>
+        <f t="shared" ref="D328:D336" si="15">100*(B328-C328)/C328</f>
         <v>1.1342962785504698</v>
       </c>
       <c r="E328">
@@ -7980,7 +7980,7 @@
         <v>2212.31</v>
       </c>
       <c r="D329">
-        <f>100*(B329-C329)/C329</f>
+        <f t="shared" si="15"/>
         <v>-3.2576808855895041E-2</v>
       </c>
       <c r="E329">
@@ -8001,7 +8001,7 @@
         <v>2212.31</v>
       </c>
       <c r="D330">
-        <f>100*(B330-C330)/C330</f>
+        <f t="shared" si="15"/>
         <v>-0.87063431435919314</v>
       </c>
       <c r="E330">
@@ -8022,7 +8022,7 @@
         <v>2212.31</v>
       </c>
       <c r="D331">
-        <f>100*(B331-C331)/C331</f>
+        <f t="shared" si="15"/>
         <v>1.1915608572035692</v>
       </c>
       <c r="E331">
@@ -8043,7 +8043,7 @@
         <v>2212.31</v>
       </c>
       <c r="D332">
-        <f>100*(B332-C332)/C332</f>
+        <f t="shared" si="15"/>
         <v>0.68783307945089511</v>
       </c>
       <c r="E332">
@@ -8064,7 +8064,7 @@
         <v>2212.31</v>
       </c>
       <c r="D333">
-        <f>100*(B333-C333)/C333</f>
+        <f t="shared" si="15"/>
         <v>1.4416406380660929</v>
       </c>
       <c r="E333">
@@ -8085,13 +8085,55 @@
         <v>2212.31</v>
       </c>
       <c r="D334">
-        <f>100*(B334-C334)/C334</f>
+        <f t="shared" si="15"/>
         <v>-3.4569748362558626E-2</v>
       </c>
       <c r="E334">
         <v>217</v>
       </c>
       <c r="F334" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="335" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A335" s="1">
+        <v>46161</v>
+      </c>
+      <c r="B335" s="2">
+        <v>2190.7586000000001</v>
+      </c>
+      <c r="C335">
+        <v>2212.31</v>
+      </c>
+      <c r="D335">
+        <f t="shared" si="15"/>
+        <v>-0.97415823279738512</v>
+      </c>
+      <c r="E335">
+        <v>217</v>
+      </c>
+      <c r="F335" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="336" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A336" s="1">
+        <v>46161</v>
+      </c>
+      <c r="B336" s="4">
+        <v>2217.7904100000001</v>
+      </c>
+      <c r="C336">
+        <v>2212.31</v>
+      </c>
+      <c r="D336">
+        <f t="shared" si="15"/>
+        <v>0.24772342031632638</v>
+      </c>
+      <c r="E336">
+        <v>217</v>
+      </c>
+      <c r="F336" t="s">
         <v>122</v>
       </c>
     </row>

</xml_diff>

<commit_message>
POWELL TA APRIL 6 6:00 BIOFAC LAST OF 24HR RUN
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48B1EBE6-2598-47EF-9A87-798C160BD7E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68296C1D-FEF4-4B1E-BEDB-5A1AFE109856}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14040" yWindow="1095" windowWidth="13425" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13695" yWindow="750" windowWidth="13425" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="123">
   <si>
     <t>Date</t>
   </si>
@@ -1256,7 +1256,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G336"/>
+  <dimension ref="A1:G337"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -7959,7 +7959,7 @@
         <v>2212.31</v>
       </c>
       <c r="D328">
-        <f t="shared" ref="D328:D336" si="15">100*(B328-C328)/C328</f>
+        <f t="shared" ref="D328:D337" si="15">100*(B328-C328)/C328</f>
         <v>1.1342962785504698</v>
       </c>
       <c r="E328">
@@ -8135,6 +8135,27 @@
       </c>
       <c r="F336" t="s">
         <v>122</v>
+      </c>
+    </row>
+    <row r="337" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A337" s="1">
+        <v>46162</v>
+      </c>
+      <c r="B337" s="2">
+        <v>2219.0449699999999</v>
+      </c>
+      <c r="C337">
+        <v>2212.31</v>
+      </c>
+      <c r="D337">
+        <f t="shared" si="15"/>
+        <v>0.30443156700462304</v>
+      </c>
+      <c r="E337">
+        <v>217</v>
+      </c>
+      <c r="F337" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MC ran KB 2026-06-27
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68296C1D-FEF4-4B1E-BEDB-5A1AFE109856}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55A08E4B-71D1-4D21-B145-41BF6A40CDBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13695" yWindow="750" windowWidth="13425" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15375" yWindow="645" windowWidth="13425" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="123">
   <si>
     <t>Date</t>
   </si>
@@ -1256,7 +1256,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G337"/>
+  <dimension ref="A1:G338"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -7959,7 +7959,7 @@
         <v>2212.31</v>
       </c>
       <c r="D328">
-        <f t="shared" ref="D328:D337" si="15">100*(B328-C328)/C328</f>
+        <f t="shared" ref="D328:D338" si="15">100*(B328-C328)/C328</f>
         <v>1.1342962785504698</v>
       </c>
       <c r="E328">
@@ -8155,6 +8155,27 @@
         <v>217</v>
       </c>
       <c r="F337" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="338" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A338" s="1">
+        <v>46204</v>
+      </c>
+      <c r="B338">
+        <v>2207.9579199999998</v>
+      </c>
+      <c r="C338">
+        <v>2212.31</v>
+      </c>
+      <c r="D338">
+        <f t="shared" si="15"/>
+        <v>-0.19672107435215294</v>
+      </c>
+      <c r="E338">
+        <v>217</v>
+      </c>
+      <c r="F338" t="s">
         <v>121</v>
       </c>
     </row>

</xml_diff>

<commit_message>
MC ran Sandy 2026/07/11
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55A08E4B-71D1-4D21-B145-41BF6A40CDBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8D31C6B-1E32-4ADC-BAAF-CD1E48087BD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15375" yWindow="645" windowWidth="13425" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15465" yWindow="645" windowWidth="13335" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="123">
   <si>
     <t>Date</t>
   </si>
@@ -1256,7 +1256,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G338"/>
+  <dimension ref="A1:G339"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -7959,7 +7959,7 @@
         <v>2212.31</v>
       </c>
       <c r="D328">
-        <f t="shared" ref="D328:D338" si="15">100*(B328-C328)/C328</f>
+        <f t="shared" ref="D328:D339" si="15">100*(B328-C328)/C328</f>
         <v>1.1342962785504698</v>
       </c>
       <c r="E328">
@@ -8176,6 +8176,27 @@
         <v>217</v>
       </c>
       <c r="F338" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="339" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A339" s="1">
+        <v>46216</v>
+      </c>
+      <c r="B339" s="4">
+        <v>2213.3171600000001</v>
+      </c>
+      <c r="C339">
+        <v>2212.31</v>
+      </c>
+      <c r="D339">
+        <f t="shared" si="15"/>
+        <v>4.5525265446529316E-2</v>
+      </c>
+      <c r="E339">
+        <v>217</v>
+      </c>
+      <c r="F339" t="s">
         <v>121</v>
       </c>
     </row>

</xml_diff>

<commit_message>
MP MARCH 18 1200 AND 2100 DATA ADD
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8D31C6B-1E32-4ADC-BAAF-CD1E48087BD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2265CEEE-E19B-477F-8342-608E7FD968F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15465" yWindow="645" windowWidth="13335" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1080" yWindow="1080" windowWidth="22965" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="126">
   <si>
     <t>Date</t>
   </si>
@@ -402,6 +402,15 @@
   </si>
   <si>
     <t>same CRM opened 05/14/2026, REDO</t>
+  </si>
+  <si>
+    <t>new CRM opened 08/27/2026</t>
+  </si>
+  <si>
+    <t>same CRM opened 08/27/2027 MP run after MC</t>
+  </si>
+  <si>
+    <t>same CRM opened 08/27/2026</t>
   </si>
 </sst>
 </file>
@@ -562,10 +571,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Lucida Console"/>
-      <family val="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="34">
@@ -924,16 +934,17 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1256,7 +1267,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G339"/>
+  <dimension ref="A1:G342"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -4812,7 +4823,7 @@
       <c r="A178" s="1">
         <v>45177</v>
       </c>
-      <c r="B178" s="2">
+      <c r="B178" s="5">
         <v>2218.4690000000001</v>
       </c>
       <c r="C178">
@@ -7175,7 +7186,7 @@
       <c r="A291" s="1">
         <v>45761</v>
       </c>
-      <c r="B291" s="4">
+      <c r="B291" s="6">
         <v>2211.8963100000001</v>
       </c>
       <c r="C291">
@@ -7196,7 +7207,7 @@
       <c r="A292" s="1">
         <v>45818</v>
       </c>
-      <c r="B292" s="4">
+      <c r="B292" s="6">
         <v>2193.6378800000002</v>
       </c>
       <c r="C292">
@@ -7217,7 +7228,7 @@
       <c r="A293" s="1">
         <v>45820</v>
       </c>
-      <c r="B293" s="4">
+      <c r="B293" s="6">
         <v>2195.2128299999999</v>
       </c>
       <c r="C293">
@@ -7238,7 +7249,7 @@
       <c r="A294" s="1">
         <v>45832</v>
       </c>
-      <c r="B294" s="4">
+      <c r="B294" s="6">
         <v>2198.7649900000001</v>
       </c>
       <c r="C294">
@@ -7259,7 +7270,7 @@
       <c r="A295" s="1">
         <v>45833</v>
       </c>
-      <c r="B295" s="4">
+      <c r="B295" s="6">
         <v>2191.2403300000001</v>
       </c>
       <c r="C295">
@@ -7280,7 +7291,7 @@
       <c r="A296" s="1">
         <v>45860</v>
       </c>
-      <c r="B296" s="4">
+      <c r="B296" s="6">
         <v>2185.3806199999999</v>
       </c>
       <c r="C296">
@@ -7301,7 +7312,7 @@
       <c r="A297" s="1">
         <v>45860</v>
       </c>
-      <c r="B297" s="4">
+      <c r="B297" s="6">
         <v>2195.7069999999999</v>
       </c>
       <c r="C297">
@@ -7322,7 +7333,7 @@
       <c r="A298" s="1">
         <v>45867</v>
       </c>
-      <c r="B298" s="4">
+      <c r="B298" s="6">
         <v>2193.57456</v>
       </c>
       <c r="C298">
@@ -7343,7 +7354,7 @@
       <c r="A299" s="1">
         <v>45868</v>
       </c>
-      <c r="B299" s="4">
+      <c r="B299" s="6">
         <v>2193.4159</v>
       </c>
       <c r="C299">
@@ -7364,7 +7375,7 @@
       <c r="A300" s="1">
         <v>45971</v>
       </c>
-      <c r="B300" s="4">
+      <c r="B300" s="6">
         <v>2177.01359</v>
       </c>
       <c r="C300">
@@ -7385,7 +7396,7 @@
       <c r="A301" s="1">
         <v>45971</v>
       </c>
-      <c r="B301" s="4">
+      <c r="B301" s="6">
         <v>2161.3153600000001</v>
       </c>
       <c r="C301">
@@ -7406,7 +7417,7 @@
       <c r="A302" s="1">
         <v>45971</v>
       </c>
-      <c r="B302" s="4">
+      <c r="B302" s="6">
         <v>2182.5608900000002</v>
       </c>
       <c r="C302">
@@ -7427,7 +7438,7 @@
       <c r="A303" s="1">
         <v>45974</v>
       </c>
-      <c r="B303" s="4">
+      <c r="B303" s="6">
         <v>2204.3165600000002</v>
       </c>
       <c r="C303">
@@ -7448,7 +7459,7 @@
       <c r="A304" s="1">
         <v>45974</v>
       </c>
-      <c r="B304" s="4">
+      <c r="B304" s="6">
         <v>2203.0845800000002</v>
       </c>
       <c r="C304">
@@ -7469,7 +7480,7 @@
       <c r="A305" s="1">
         <v>45985</v>
       </c>
-      <c r="B305" s="4">
+      <c r="B305" s="6">
         <v>2196.3349600000001</v>
       </c>
       <c r="C305">
@@ -7490,7 +7501,7 @@
       <c r="A306" s="1">
         <v>45985</v>
       </c>
-      <c r="B306" s="4">
+      <c r="B306" s="6">
         <v>2204.1925099999999</v>
       </c>
       <c r="C306">
@@ -7511,7 +7522,7 @@
       <c r="A307" s="1">
         <v>46062</v>
       </c>
-      <c r="B307" s="4">
+      <c r="B307" s="6">
         <v>2262.82393</v>
       </c>
       <c r="C307">
@@ -7532,7 +7543,7 @@
       <c r="A308" s="1">
         <v>46076</v>
       </c>
-      <c r="B308" s="4">
+      <c r="B308" s="6">
         <v>2192.07897</v>
       </c>
       <c r="C308">
@@ -7553,7 +7564,7 @@
       <c r="A309" s="1">
         <v>46077</v>
       </c>
-      <c r="B309" s="4">
+      <c r="B309" s="6">
         <v>2202.3117900000002</v>
       </c>
       <c r="C309">
@@ -7574,7 +7585,7 @@
       <c r="A310" s="1">
         <v>46089</v>
       </c>
-      <c r="B310" s="4">
+      <c r="B310" s="6">
         <v>2207.98432</v>
       </c>
       <c r="C310">
@@ -7595,7 +7606,7 @@
       <c r="A311" s="1">
         <v>46089</v>
       </c>
-      <c r="B311" s="4">
+      <c r="B311" s="6">
         <v>2203.7444399999999</v>
       </c>
       <c r="C311">
@@ -7616,7 +7627,7 @@
       <c r="A312" s="1">
         <v>46094</v>
       </c>
-      <c r="B312" s="4">
+      <c r="B312" s="6">
         <v>2209.9749200000001</v>
       </c>
       <c r="C312">
@@ -7637,7 +7648,7 @@
       <c r="A313" s="1">
         <v>46096</v>
       </c>
-      <c r="B313" s="4">
+      <c r="B313" s="6">
         <v>2195.19785</v>
       </c>
       <c r="C313">
@@ -7658,7 +7669,7 @@
       <c r="A314" s="1">
         <v>46096</v>
       </c>
-      <c r="B314" s="4">
+      <c r="B314" s="6">
         <v>2222.4642699999999</v>
       </c>
       <c r="C314">
@@ -7679,7 +7690,7 @@
       <c r="A315" s="1">
         <v>46098</v>
       </c>
-      <c r="B315" s="4">
+      <c r="B315" s="6">
         <v>2209.22534</v>
       </c>
       <c r="C315">
@@ -7700,7 +7711,7 @@
       <c r="A316" s="1">
         <v>46100</v>
       </c>
-      <c r="B316" s="4">
+      <c r="B316" s="6">
         <v>2203.9237600000001</v>
       </c>
       <c r="C316">
@@ -7721,7 +7732,7 @@
       <c r="A317" s="1">
         <v>46101</v>
       </c>
-      <c r="B317" s="4">
+      <c r="B317" s="6">
         <v>2248.6597999999999</v>
       </c>
       <c r="C317">
@@ -7742,7 +7753,7 @@
       <c r="A318" s="1">
         <v>46101</v>
       </c>
-      <c r="B318" s="4">
+      <c r="B318" s="6">
         <v>2210.7517400000002</v>
       </c>
       <c r="C318">
@@ -7763,7 +7774,7 @@
       <c r="A319" s="1">
         <v>46108</v>
       </c>
-      <c r="B319" s="4">
+      <c r="B319" s="6">
         <v>2205.7238900000002</v>
       </c>
       <c r="C319">
@@ -7805,7 +7816,7 @@
       <c r="A321" s="1">
         <v>46133</v>
       </c>
-      <c r="B321" s="4">
+      <c r="B321" s="6">
         <v>2200.2290600000001</v>
       </c>
       <c r="C321">
@@ -7826,7 +7837,7 @@
       <c r="A322" s="1">
         <v>46146</v>
       </c>
-      <c r="B322" s="2">
+      <c r="B322" s="5">
         <v>2209.3617300000001</v>
       </c>
       <c r="C322">
@@ -7847,7 +7858,7 @@
       <c r="A323" s="1">
         <v>46146</v>
       </c>
-      <c r="B323" s="2">
+      <c r="B323" s="5">
         <v>2211.4530599999998</v>
       </c>
       <c r="C323">
@@ -7868,7 +7879,7 @@
       <c r="A324" s="1">
         <v>46146</v>
       </c>
-      <c r="B324" s="2">
+      <c r="B324" s="5">
         <v>2207.8857499999999</v>
       </c>
       <c r="C324">
@@ -7889,7 +7900,7 @@
       <c r="A325" s="1">
         <v>46147</v>
       </c>
-      <c r="B325" s="2">
+      <c r="B325" s="5">
         <v>2218.4741899999999</v>
       </c>
       <c r="C325">
@@ -7910,7 +7921,7 @@
       <c r="A326" s="1">
         <v>46149</v>
       </c>
-      <c r="B326" s="4">
+      <c r="B326" s="6">
         <v>2209.5682700000002</v>
       </c>
       <c r="C326">
@@ -7931,7 +7942,7 @@
       <c r="A327" s="1">
         <v>46149</v>
       </c>
-      <c r="B327" s="4">
+      <c r="B327" s="6">
         <v>2211.0061500000002</v>
       </c>
       <c r="C327">
@@ -7952,14 +7963,14 @@
       <c r="A328" s="1">
         <v>46150</v>
       </c>
-      <c r="B328" s="5">
+      <c r="B328" s="4">
         <v>2237.4041499999998</v>
       </c>
       <c r="C328">
         <v>2212.31</v>
       </c>
       <c r="D328">
-        <f t="shared" ref="D328:D339" si="15">100*(B328-C328)/C328</f>
+        <f t="shared" ref="D328:D340" si="15">100*(B328-C328)/C328</f>
         <v>1.1342962785504698</v>
       </c>
       <c r="E328">
@@ -7973,7 +7984,7 @@
       <c r="A329" s="1">
         <v>46150</v>
       </c>
-      <c r="B329" s="2">
+      <c r="B329" s="5">
         <v>2211.5893000000001</v>
       </c>
       <c r="C329">
@@ -7994,7 +8005,7 @@
       <c r="A330" s="1">
         <v>46154</v>
       </c>
-      <c r="B330" s="2">
+      <c r="B330" s="5">
         <v>2193.0488700000001</v>
       </c>
       <c r="C330">
@@ -8015,7 +8026,7 @@
       <c r="A331" s="1">
         <v>46156</v>
       </c>
-      <c r="B331" s="2">
+      <c r="B331" s="5">
         <v>2238.6710200000002</v>
       </c>
       <c r="C331">
@@ -8036,7 +8047,7 @@
       <c r="A332" s="1">
         <v>46156</v>
       </c>
-      <c r="B332" s="2">
+      <c r="B332" s="5">
         <v>2227.527</v>
       </c>
       <c r="C332">
@@ -8057,7 +8068,7 @@
       <c r="A333" s="1">
         <v>46157</v>
       </c>
-      <c r="B333" s="2">
+      <c r="B333" s="5">
         <v>2244.2035599999999</v>
       </c>
       <c r="C333">
@@ -8078,7 +8089,7 @@
       <c r="A334" s="1">
         <v>46157</v>
       </c>
-      <c r="B334" s="2">
+      <c r="B334" s="5">
         <v>2211.5452100000002</v>
       </c>
       <c r="C334">
@@ -8099,7 +8110,7 @@
       <c r="A335" s="1">
         <v>46161</v>
       </c>
-      <c r="B335" s="2">
+      <c r="B335" s="5">
         <v>2190.7586000000001</v>
       </c>
       <c r="C335">
@@ -8120,7 +8131,7 @@
       <c r="A336" s="1">
         <v>46161</v>
       </c>
-      <c r="B336" s="4">
+      <c r="B336" s="6">
         <v>2217.7904100000001</v>
       </c>
       <c r="C336">
@@ -8141,7 +8152,7 @@
       <c r="A337" s="1">
         <v>46162</v>
       </c>
-      <c r="B337" s="2">
+      <c r="B337" s="5">
         <v>2219.0449699999999</v>
       </c>
       <c r="C337">
@@ -8183,7 +8194,7 @@
       <c r="A339" s="1">
         <v>46216</v>
       </c>
-      <c r="B339" s="4">
+      <c r="B339" s="6">
         <v>2213.3171600000001</v>
       </c>
       <c r="C339">
@@ -8198,6 +8209,69 @@
       </c>
       <c r="F339" t="s">
         <v>121</v>
+      </c>
+    </row>
+    <row r="340" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A340" s="1">
+        <v>46261</v>
+      </c>
+      <c r="B340">
+        <v>2215.8625400000001</v>
+      </c>
+      <c r="C340">
+        <v>2212.31</v>
+      </c>
+      <c r="D340">
+        <f t="shared" si="15"/>
+        <v>0.16058056963084449</v>
+      </c>
+      <c r="E340">
+        <v>217</v>
+      </c>
+      <c r="F340" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="341" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A341" s="1">
+        <v>46261</v>
+      </c>
+      <c r="B341" s="2">
+        <v>2211.2017099999998</v>
+      </c>
+      <c r="C341">
+        <v>2212.31</v>
+      </c>
+      <c r="D341">
+        <f>100*(B341-C341)/C341</f>
+        <v>-5.0096505462621628E-2</v>
+      </c>
+      <c r="E341">
+        <v>217</v>
+      </c>
+      <c r="F341" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="342" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A342" s="1">
+        <v>46265</v>
+      </c>
+      <c r="B342" s="2">
+        <v>2222.3018499999998</v>
+      </c>
+      <c r="C342">
+        <v>2212.31</v>
+      </c>
+      <c r="D342">
+        <f>100*(B342-C342)/C342</f>
+        <v>0.45164782512396029</v>
+      </c>
+      <c r="E342">
+        <v>217</v>
+      </c>
+      <c r="F342" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
POWELL 10 MARCH 2100 BIOFAC
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2265CEEE-E19B-477F-8342-608E7FD968F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C36A0740-7FD0-41BD-8531-BA1616953994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1080" windowWidth="22965" windowHeight="14100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15825" yWindow="105" windowWidth="12975" windowHeight="15135" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="126">
   <si>
     <t>Date</t>
   </si>
@@ -1267,7 +1267,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G342"/>
+  <dimension ref="A1:G343"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -8274,6 +8274,27 @@
         <v>125</v>
       </c>
     </row>
+    <row r="343" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A343" s="1">
+        <v>46266</v>
+      </c>
+      <c r="B343" s="2">
+        <v>2231.89662</v>
+      </c>
+      <c r="C343">
+        <v>2212.31</v>
+      </c>
+      <c r="D343">
+        <f>100*(B343-C343)/C343</f>
+        <v>0.88534699025001196</v>
+      </c>
+      <c r="E343">
+        <v>217</v>
+      </c>
+      <c r="F343" t="s">
+        <v>125</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
MP FIRST 1/2 OF BIOFAC MARCH10 12PM
</commit_message>
<xml_diff>
--- a/Data/CRMAccuracyData.xlsx
+++ b/Data/CRMAccuracyData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Titrator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C36A0740-7FD0-41BD-8531-BA1616953994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63CE21A9-BEA5-4614-A5AE-F76E0914976C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15825" yWindow="105" windowWidth="12975" windowHeight="15135" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15330" yWindow="45" windowWidth="12975" windowHeight="15135" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRMAccuracyData" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="127">
   <si>
     <t>Date</t>
   </si>
@@ -411,6 +411,9 @@
   </si>
   <si>
     <t>same CRM opened 08/27/2026</t>
+  </si>
+  <si>
+    <t>same CRM opened 08/27/2026, REDID</t>
   </si>
 </sst>
 </file>
@@ -1267,7 +1270,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G343"/>
+  <dimension ref="A1:G345"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -8295,6 +8298,48 @@
         <v>125</v>
       </c>
     </row>
+    <row r="344" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A344" s="1">
+        <v>46266</v>
+      </c>
+      <c r="B344" s="2">
+        <v>2220.8210899999999</v>
+      </c>
+      <c r="C344">
+        <v>2212.31</v>
+      </c>
+      <c r="D344">
+        <f>100*(B344-C344)/C344</f>
+        <v>0.38471507157676671</v>
+      </c>
+      <c r="E344">
+        <v>217</v>
+      </c>
+      <c r="F344" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="345" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A345" s="1">
+        <v>46267</v>
+      </c>
+      <c r="B345" s="2">
+        <v>2211.1793400000001</v>
+      </c>
+      <c r="C345">
+        <v>2212.31</v>
+      </c>
+      <c r="D345">
+        <f>100*(B345-C345)/C345</f>
+        <v>-5.1107665743038141E-2</v>
+      </c>
+      <c r="E345">
+        <v>217</v>
+      </c>
+      <c r="F345" t="s">
+        <v>125</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>